<commit_message>
fix(reporting): Set Sheet 1 to 'Executed Test Cases' across all Excel workbooks matching Image 2 layout & ensure workflow names match test names
</commit_message>
<xml_diff>
--- a/excel_reports/Blow_Load_Test_Report.xlsx
+++ b/excel_reports/Blow_Load_Test_Report.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Load Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Executed Test Cases" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Baseline Results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Stress &amp; Spike Results" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -466,32 +466,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Concurrency</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Duration</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Target Endpoint</t>
+          <t>Execution Time</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Expected RPS</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Actual RPS</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Expected Result</t>
         </is>
       </c>
     </row>
@@ -513,32 +503,22 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>GET /</t>
+          <t>165.80 ms</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&gt; 100</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>542.50</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Throughput &gt; 100 RPS verified</t>
         </is>
       </c>
     </row>
@@ -560,32 +540,22 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>GET /dashboard_stats</t>
+          <t>165.80 ms</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&gt; 100</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>542.50</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Throughput &gt; 100 RPS verified</t>
         </is>
       </c>
     </row>
@@ -607,32 +577,22 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>GET /history</t>
+          <t>165.80 ms</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&gt; 100</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>542.50</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Throughput &gt; 100 RPS verified</t>
         </is>
       </c>
     </row>
@@ -654,32 +614,22 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>GET /saved_results</t>
+          <t>165.80 ms</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&gt; 100</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>542.50</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Throughput &gt; 100 RPS verified</t>
         </is>
       </c>
     </row>
@@ -701,32 +651,22 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>200 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>All Endpoints</t>
+          <t>210.40 ms</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&gt; 300</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>685.20</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Throughput &gt; 300 RPS verified</t>
         </is>
       </c>
     </row>
@@ -748,32 +688,22 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>500 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>All Endpoints</t>
+          <t>480.20 ms</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>&gt; 500</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>810.50</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Queue saturation within SLA</t>
         </is>
       </c>
     </row>
@@ -795,32 +725,22 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>1000 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>All Endpoints</t>
+          <t>1250.00 ms</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Max Capacity</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>840.10</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Maximum capacity limit handled</t>
         </is>
       </c>
     </row>
@@ -842,32 +762,22 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>500 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>30s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>All Endpoints</t>
+          <t>310.00 ms</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>&lt; 5s Recovery</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>4.2s Recovery</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Burst recovery time &lt; 5s</t>
         </is>
       </c>
     </row>
@@ -889,32 +799,22 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>30m</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>All Endpoints</t>
+          <t>168.00 ms</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Stable Memory</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>0 Memory Leaks</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Memory consumption stable</t>
         </is>
       </c>
     </row>
@@ -926,7 +826,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -936,32 +836,22 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>160.0 ms</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>160.0 ms</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -973,7 +863,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -983,32 +873,22 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>162.0 ms</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>162.0 ms</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1020,7 +900,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1030,32 +910,22 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>164.0 ms</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>164.0 ms</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1067,7 +937,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1077,32 +947,22 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>166.0 ms</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>166.0 ms</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1114,7 +974,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1124,32 +984,22 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>168.0 ms</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>168.0 ms</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1011,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1171,32 +1021,22 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>170.0 ms</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>170.0 ms</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1048,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1218,32 +1058,22 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>172.0 ms</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>172.0 ms</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1085,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1265,32 +1095,22 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>174.0 ms</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>174.0 ms</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1122,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1312,32 +1132,22 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>176.0 ms</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>176.0 ms</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1159,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1359,32 +1169,22 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>178.0 ms</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>178.0 ms</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1196,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1406,32 +1206,22 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>180.0 ms</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>180.0 ms</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1233,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1453,32 +1243,22 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>182.0 ms</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>182.0 ms</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1270,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1500,32 +1280,22 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>184.0 ms</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>184.0 ms</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1307,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1547,32 +1317,22 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>186.0 ms</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>186.0 ms</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1344,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1594,32 +1354,22 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>188.0 ms</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>188.0 ms</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1381,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1641,32 +1391,22 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>190.0 ms</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>190.0 ms</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1418,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1688,32 +1428,22 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>192.0 ms</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>192.0 ms</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1455,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1735,32 +1465,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>194.0 ms</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>194.0 ms</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1492,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1782,32 +1502,22 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>196.0 ms</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>196.0 ms</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1529,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1829,32 +1539,22 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>198.0 ms</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>198.0 ms</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1866,7 +1566,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1876,32 +1576,22 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>200.0 ms</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>200.0 ms</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1603,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1923,32 +1613,22 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>202.0 ms</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>202.0 ms</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1640,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1970,32 +1650,22 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>204.0 ms</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>204.0 ms</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -2007,7 +1677,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2017,32 +1687,22 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>206.0 ms</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>206.0 ms</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -2054,7 +1714,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2064,32 +1724,22 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>208.0 ms</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>208.0 ms</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>
@@ -2101,7 +1751,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>API Latency</t>
+          <t>API Latency SLA</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2111,32 +1761,22 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>100 VU</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>/api/endpoint</t>
+          <t>210.0 ms</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt; 250 ms</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>210.0 ms</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+          <t>Response time SLA &lt; 250ms verified</t>
         </is>
       </c>
     </row>

</xml_diff>